<commit_message>
add reference for HCFE-235da2
</commit_message>
<xml_diff>
--- a/tools/value_references.xlsx
+++ b/tools/value_references.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eearp\Desktop\anesthesia\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\eearp\code\anaesthetic-project\tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{98F0ED56-3409-4CAB-8A5A-D858931DB8A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E11319B6-6658-4240-AAB2-C010F6A5AFA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{F8D153B5-466C-478D-A3C3-E300523FCDFB}"/>
   </bookViews>
@@ -114,7 +114,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -125,6 +125,14 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -147,14 +155,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -624,7 +635,7 @@
         <v>15</v>
       </c>
       <c r="D7" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E7" t="s">
         <v>16</v>
@@ -702,7 +713,7 @@
       <c r="A13" t="s">
         <v>12</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="2" t="s">
         <v>14</v>
       </c>
     </row>
@@ -723,6 +734,9 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B13" r:id="rId1" xr:uid="{80051077-AD4D-4B9B-A94D-778898DBACDB}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>